<commit_message>
feat: complete Phase 2 advanced multi-solution suite (MA, OK, TL, WA, Python), vision problem parser, and modern web dashboard
</commit_message>
<xml_diff>
--- a/problems_summary.xlsx
+++ b/problems_summary.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -882,6 +882,53 @@
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>domino-piling</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>https://codeforces.com/problemset/problem/50/A</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>577496</v>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>https://polygon.codeforces.com/p577496/domino-piling</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>https://polygon.codeforces.com/p577496/luatgay/domino-piling</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>1456787</v>
+      </c>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-23 21:48:57</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -906,6 +953,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId24"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: generator cpp + polygon freemarker script, marisaoj scraper, retry/backoff improvements, lcmp checker, utf8 cli fix
</commit_message>
<xml_diff>
--- a/problems_summary.xlsx
+++ b/problems_summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Problems" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Problems" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -775,7 +775,7 @@
         </is>
       </c>
       <c r="H6" s="2" t="n">
-        <v>1456226</v>
+        <v>1461279</v>
       </c>
       <c r="I6" s="6" t="inlineStr">
         <is>
@@ -929,6 +929,205 @@
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>creating-abbreviations</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>https://codeforces.com/problemset/problem/2257/A</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>578710</v>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>https://polygon.codeforces.com/p578710/creating-abbreviations</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>https://polygon.codeforces.com/p578710/luatgay/creating-abbreviations</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 23:13:46</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>Failed calling problem.saveSolution after 5 attempts: HTTP 400: file: C:/Programs/mingw-w64-7/bin/../lib/gcc/i686-w64-mingw32/7.3.0/../../../../i686-w64-mingw32/lib/../lib\libmingw32.a(lib32_libmingw32_a-crt0_c.o):crt0_c.c:(.text.startup+0x39): undefined reference to `WinMain@16'
+collect2.exe: error: ld returned 1 exit sta</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>the-best-card</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>https://codeforces.com/problemset/problem/2253/A</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>578750</v>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>https://polygon.codeforces.com/p578750/the-best-card</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>https://polygon.codeforces.com/p578750/luatgay/the-best-card</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>1460310</v>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-28 02:04:08</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>Polygon package build failed on package 1460310. Verification checks did not pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>who-watches-the-watchpig</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>https://codeforces.com/contest/2245/problem/A</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>578756</v>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>https://polygon.codeforces.com/p578756/who-watches-the-watchpig</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>https://polygon.codeforces.com/p578756/luatgay/who-watches-the-watchpig</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>1460324</v>
+      </c>
+      <c r="I12" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-28 03:33:56</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>divide-and-conquer</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>https://codeforces.com/problemset/problem/2241/A</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>579119</v>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>https://polygon.codeforces.com/p579119/divide-and-conquer</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>https://polygon.codeforces.com/p579119/luatgay/divide-and-conquer</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>1461304</v>
+      </c>
+      <c r="I13" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-29 09:45:08</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -956,6 +1155,18 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId36"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: complete 10-step sequential pipeline with subtasks and resilience
</commit_message>
<xml_diff>
--- a/problems_summary.xlsx
+++ b/problems_summary.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -490,11 +490,13 @@
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="42" customWidth="1" min="5" max="5"/>
     <col width="46" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="35" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="23" customWidth="1" min="10" max="10"/>
-    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="23" customWidth="1" min="12" max="12"/>
+    <col width="30" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -530,25 +532,35 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Số Lượng Test</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Subtasks &amp; Điểm</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>Trạng Thái Package</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Package ID</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Sẵn Sàng Import CF</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Thời Gian Tạo</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Ghi Chú / Lỗi</t>
         </is>
@@ -560,46 +572,62 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>evanescent</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>https://codeforces.com/problemset/problem/2254/B</t>
+          <t>https://codeforces.com/problemset/problem/4/A</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>577293</v>
+        <v>0</v>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>https://polygon.codeforces.com/p577293/evanescent</t>
+          <t>https://polygon.codeforces.com/p0/Unknown</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>https://polygon.codeforces.com/p577293/luatgay/evanescent</t>
-        </is>
-      </c>
-      <c r="G2" s="5" t="inlineStr">
+          <t>https://polygon.codeforces.com/p0/Unknown</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
         <is>
           <t>FAILED</t>
         </is>
       </c>
-      <c r="H2" s="2" t="n">
-        <v>1456133</v>
-      </c>
-      <c r="I2" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 09:42:00</t>
-        </is>
-      </c>
-      <c r="K2" s="3" t="inlineStr"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18 07:53:44</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>cannot access local variable 's' where it is not associated with a value</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -607,328 +635,54 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>hot-potatoes-at-the-fairy-ware</t>
+          <t>watermelon</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>https://codeforces.com/contest/2256/problem/C</t>
+          <t>https://codeforces.com/problemset/problem/4/A</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>577252</v>
+        <v>577334</v>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>https://polygon.codeforces.com/p577252/hot-potatoes-at-the-fairy-ware</t>
+          <t>https://polygon.codeforces.com/p577334/watermelon</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>https://polygon.codeforces.com/p577252/luatgay/hot-potatoes-at-the-fairy-ware</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="n">
-        <v>1455816</v>
-      </c>
-      <c r="I3" s="6" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-23 10:02:06</t>
-        </is>
-      </c>
-      <c r="K3" s="3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>watermelon</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>https://codeforces.com/problemset/problem/4/A</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="n">
-        <v>577334</v>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>https://polygon.codeforces.com/p577334/watermelon</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
           <t>https://polygon.codeforces.com/p577334/luatgay/watermelon</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>READY</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="n">
-        <v>1459663</v>
-      </c>
-      <c r="I4" s="6" t="inlineStr">
+      <c r="G3" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Subtask 1 (30.0 pts: 6 tests), Subtask 2 (30.0 pts: 6 tests), Subtask 3 (40.0 pts: 8 tests)</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>RUNNING</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>1518969</v>
+      </c>
+      <c r="K3" s="6" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-23 12:21:26</t>
-        </is>
-      </c>
-      <c r="K4" s="3" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>boss-fight</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>https://codeforces.com/problemset/problem/2252/A</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="n">
-        <v>577335</v>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>https://polygon.codeforces.com/p577335/boss-fight</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>https://polygon.codeforces.com/p577335/luatgay/boss-fight</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>READY</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="n">
-        <v>1456213</v>
-      </c>
-      <c r="I5" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-23 12:28:11</t>
-        </is>
-      </c>
-      <c r="K5" s="3" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>theatre-square</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>https://codeforces.com/problemset/problem/1/A</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="n">
-        <v>577343</v>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>https://polygon.codeforces.com/p577343/theatre-square</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>https://polygon.codeforces.com/p577343/luatgay/theatre-square</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>READY</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>1456226</v>
-      </c>
-      <c r="I6" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-23 12:50:37</t>
-        </is>
-      </c>
-      <c r="K6" s="3" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>way-too-long-words</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>https://codeforces.com/problemset/problem/71/A</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="n">
-        <v>577349</v>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>https://polygon.codeforces.com/p577349/way-too-long-words</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>https://polygon.codeforces.com/p577349/luatgay/way-too-long-words</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>READY</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="n">
-        <v>1456234</v>
-      </c>
-      <c r="I7" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-23 13:12:01</t>
-        </is>
-      </c>
-      <c r="K7" s="3" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>next-round</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>https://codeforces.com/problemset/problem/158/A</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="n">
-        <v>577351</v>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>https://polygon.codeforces.com/p577351/next-round</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>https://polygon.codeforces.com/p577351/luatgay/next-round</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>READY</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="n">
-        <v>1456253</v>
-      </c>
-      <c r="I8" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-23 13:34:06</t>
-        </is>
-      </c>
-      <c r="K8" s="3" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>domino-piling</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>https://codeforces.com/problemset/problem/50/A</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="n">
-        <v>577496</v>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>https://polygon.codeforces.com/p577496/domino-piling</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>https://polygon.codeforces.com/p577496/luatgay/domino-piling</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>READY</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="n">
-        <v>1456787</v>
-      </c>
-      <c r="I9" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-23 21:48:57</t>
-        </is>
-      </c>
-      <c r="K9" s="3" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18 10:35:54</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -938,24 +692,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId24"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: resolve checker_type NameError, remove blocking PolygonAPIError retries, optimize timeout handling
</commit_message>
<xml_diff>
--- a/problems_summary.xlsx
+++ b/problems_summary.xlsx
@@ -615,7 +615,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>PENDING</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t>cannot access local variable 's' where it is not associated with a value</t>
+          <t>name 'checker_type' is not defined</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: optimize package retry loop and reduce save file timeouts to avoid freezes
</commit_message>
<xml_diff>
--- a/problems_summary.xlsx
+++ b/problems_summary.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -684,6 +684,61 @@
       </c>
       <c r="M3" s="3" t="inlineStr"/>
     </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>way-too-long-words</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>https://codeforces.com/problemset/problem/71/A</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>577349</v>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>https://polygon.codeforces.com/p577349/way-too-long-words</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>https://polygon.codeforces.com/p577349/luatgay/way-too-long-words</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Subtask 1 (30.0 pts: 6 tests), Subtask 2 (30.0 pts: 6 tests), Subtask 3 (40.0 pts: 8 tests)</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>RUNNING</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>1519019</v>
+      </c>
+      <c r="K4" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18 11:38:14</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
@@ -692,6 +747,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: update problems_summary with verified problem 158A next-round
</commit_message>
<xml_diff>
--- a/problems_summary.xlsx
+++ b/problems_summary.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -739,6 +739,61 @@
       </c>
       <c r="M4" s="3" t="inlineStr"/>
     </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>next-round</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>https://codeforces.com/problemset/problem/158/A</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>577351</v>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>https://polygon.codeforces.com/p577351/next-round</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>https://polygon.codeforces.com/p577351/luatgay/next-round</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Subtask 1 (30.0 pts: 6 tests), Subtask 2 (30.0 pts: 6 tests), Subtask 3 (40.0 pts: 8 tests)</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>RUNNING</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>1519022</v>
+      </c>
+      <c r="K5" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18 11:50:05</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
@@ -750,6 +805,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: optimize pipeline speed, non-blocking Polygon upload, and Gemini Flash upgrade
</commit_message>
<xml_diff>
--- a/problems_summary.xlsx
+++ b/problems_summary.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -794,6 +794,63 @@
       </c>
       <c r="M5" s="3" t="inlineStr"/>
     </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>sausage-bank</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>https://codeforces.com/problemset/problem/2269/A</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>606627</v>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>https://polygon.codeforces.com/p606627/sausage-bank</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>https://polygon.codeforces.com/p606627/luatgay/sausage-bank</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Subtask 1 (30.0 pts: 4 tests), Subtask 2 (30.0 pts: 4 tests), Subtask 3 (40.0 pts: 7 tests)</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>QUEUED_ON_POLYGON</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K6" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18 13:46:04</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
@@ -808,6 +865,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId15"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: record verified run for problem 1850A To My Critics
</commit_message>
<xml_diff>
--- a/problems_summary.xlsx
+++ b/problems_summary.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -851,6 +851,63 @@
       </c>
       <c r="M6" s="3" t="inlineStr"/>
     </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>to-my-critics</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>https://codeforces.com/problemset/problem/1850/A</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>606645</v>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>https://polygon.codeforces.com/p606645/to-my-critics</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>https://polygon.codeforces.com/p606645/luatgay/to-my-critics</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Subtask 1 (30.0 pts: 4 tests), Subtask 2 (30.0 pts: 4 tests), Subtask 3 (40.0 pts: 7 tests)</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>QUEUED_ON_POLYGON</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K7" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18 13:53:26</t>
+        </is>
+      </c>
+      <c r="M7" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
@@ -868,6 +925,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId18"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: VNOJ PDF scraper, Polygon direct test upload with subtasks, and codeforces access
</commit_message>
<xml_diff>
--- a/problems_summary.xlsx
+++ b/problems_summary.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -907,6 +907,61 @@
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>https://oj.vnoi.info/problem/fc020_accepted</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>606912</v>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>https://polygon.codeforces.com/p606912/accepted</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>https://polygon.codeforces.com/p606912/luatgay/accepted</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Subtask 1 (30.0 pts: 4 tests), Subtask 2 (30.0 pts: 4 tests), Subtask 3 (40.0 pts: 7 tests)</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>1519634</v>
+      </c>
+      <c r="K8" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18 22:38:19</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -928,6 +983,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId21"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>